<commit_message>
Documento de salida de IDX y IDTR
</commit_message>
<xml_diff>
--- a/Proyecto/output/IDTR.xlsx
+++ b/Proyecto/output/IDTR.xlsx
@@ -371,7 +371,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>77.5763143099942</v>
+        <v>74.79614559726997</v>
       </c>
     </row>
     <row r="3">
@@ -379,7 +379,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>43.46873576924303</v>
+        <v>41.30558097717306</v>
       </c>
     </row>
     <row r="4">
@@ -387,7 +387,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>56.07469245263631</v>
+        <v>51.00981695659306</v>
       </c>
     </row>
     <row r="5">
@@ -395,7 +395,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>36.32653065056311</v>
+        <v>29.57126028809783</v>
       </c>
     </row>
     <row r="6">
@@ -403,7 +403,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>48.67875697566016</v>
+        <v>44.23266577596338</v>
       </c>
     </row>
     <row r="7">
@@ -411,7 +411,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>38.76837219974244</v>
+        <v>34.94252452913167</v>
       </c>
     </row>
     <row r="8">
@@ -419,7 +419,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>41.42168746568976</v>
+        <v>33.36345386605302</v>
       </c>
     </row>
     <row r="9">
@@ -427,7 +427,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>32.23415067674652</v>
+        <v>26.41597868272162</v>
       </c>
     </row>
     <row r="10">
@@ -435,7 +435,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>50.20779580125781</v>
+        <v>44.85204815803266</v>
       </c>
     </row>
     <row r="11">
@@ -443,7 +443,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>36.1716595263226</v>
+        <v>30.02307573929184</v>
       </c>
     </row>
     <row r="12">
@@ -451,7 +451,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>38.64741625203513</v>
+        <v>33.34656354424878</v>
       </c>
     </row>
     <row r="13">
@@ -459,7 +459,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>29.82769153100705</v>
+        <v>23.31782332578931</v>
       </c>
     </row>
     <row r="14">
@@ -467,7 +467,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>30.65826673287299</v>
+        <v>23.63624745954707</v>
       </c>
     </row>
     <row r="15">
@@ -475,7 +475,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>23.09928400254126</v>
+        <v>17.70549860707237</v>
       </c>
     </row>
     <row r="16">
@@ -483,7 +483,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>29.05908232083928</v>
+        <v>22.55416731980755</v>
       </c>
     </row>
     <row r="17">
@@ -491,7 +491,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>14.07076961023218</v>
+        <v>11.12364641310098</v>
       </c>
     </row>
     <row r="18">
@@ -499,7 +499,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>37.50613219681414</v>
+        <v>33.38613861179443</v>
       </c>
     </row>
     <row r="19">
@@ -507,7 +507,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>39.21955660882178</v>
+        <v>35.45981736861773</v>
       </c>
     </row>
     <row r="20">
@@ -515,7 +515,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>41.53529157874383</v>
+        <v>37.3084916789695</v>
       </c>
     </row>
     <row r="21">
@@ -523,7 +523,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>34.2299398334452</v>
+        <v>28.74066745380418</v>
       </c>
     </row>
     <row r="22">
@@ -531,7 +531,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>37.70730246307081</v>
+        <v>30.42193180291855</v>
       </c>
     </row>
     <row r="23">
@@ -539,7 +539,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>41.69458479267256</v>
+        <v>37.46395630275696</v>
       </c>
     </row>
   </sheetData>

</xml_diff>